<commit_message>
prep for env intl
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/Outputs/Tables/T1.xlsx
+++ b/Outputs/Tables/T1.xlsx
@@ -17,16 +17,16 @@
     <t xml:space="preserve">Variable: Subcategory</t>
   </si>
   <si>
-    <t xml:space="preserve">Follicularᵃ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FV-PTCᵃ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Papillaryᵃ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Totalᵃ</t>
+    <t xml:space="preserve">Follicular†</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IEFVPTC†</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Papillary†</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total†</t>
   </si>
   <si>
     <t xml:space="preserve">Mean Age (Years)</t>
@@ -65,7 +65,7 @@
     <t xml:space="preserve">2 (10%)</t>
   </si>
   <si>
-    <t xml:space="preserve">-</t>
+    <t xml:space="preserve">–</t>
   </si>
   <si>
     <t xml:space="preserve">2 (3%)</t>
@@ -107,7 +107,7 @@
     <t xml:space="preserve">7 (12%)</t>
   </si>
   <si>
-    <t xml:space="preserve">ᵃ All values displayed as mean ± SD for ratio continuous variables or n (%) for dichotomous categorical variables. Percentages for the variant columns were calculated in respect to total patients within a variant (i.e., within column), and percentages for the total column was calculated in respect to the population total.</t>
+    <t xml:space="preserve">† All values displayed as mean ± SD for ratio continuous variables or n (%) for dichotomous categorical variables. Percentages for the variant columns were calculated in respect to total patients within a variant (i.e., within column), and percentages for the total column was calculated in respect to the population total.</t>
   </si>
 </sst>
 </file>

</xml_diff>